<commit_message>
Make This_Weeks_Picks.xlsx an append-only running history
write_excel() now loads and appends to the existing workbook instead of
overwriting it each run, since dedupe() already guarantees no listing is
ever scored twice. Adds a Date Found column, and migrates the existing
file (written under the old overwrite-each-run schema) by backfilling
dates from state.json.
</commit_message>
<xml_diff>
--- a/This_Weeks_Picks.xlsx
+++ b/This_Weeks_Picks.xlsx
@@ -424,44 +424,50 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F15"/>
+  <dimension ref="A1:G15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="45" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="55" customWidth="1" min="5" max="5"/>
-    <col width="30" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="45" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="55" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
+          <t>Date Found</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
           <t>Title</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Organization/Source</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>URL</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Match Score</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Legal Work Flag</t>
         </is>
@@ -470,28 +476,33 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
           <t>Digital Content Creation Support for UNFPA Campaigns</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>UNFPA - United Nations Population Fund</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="D2" t="inlineStr">
         <is>
           <t>https://untalent.org/jobs/digital-content-creation-support-for-unfpa-campaigns-1</t>
         </is>
       </c>
-      <c r="D2" t="n">
+      <c r="E2" t="n">
         <v>0.55</v>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>Digital content creation for UNFPA campaigns aligns well with core skills (video production, social-first storytelling, humanitarian content) but title/location/contract type are unclear, and it may be a UN consultancy which is excluded if Switzerland-based.</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>Location not specified; if UN consultancy is based in Switzerland, this would be excluded per candidate preferences.</t>
         </is>
@@ -500,28 +511,33 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
           <t>Digital Content Creation Support for UNFPA Campaigns</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="C3" t="inlineStr">
         <is>
           <t>UNFPA - United Nations Population Fund</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="D3" t="inlineStr">
         <is>
           <t>https://untalent.org/jobs/digital-content-creation-support-for-unfpa-campaigns</t>
         </is>
       </c>
-      <c r="D3" t="n">
+      <c r="E3" t="n">
         <v>0.55</v>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t>Digital content creation for UNFPA campaigns aligns well with core skills (video production, social-first storytelling, humanitarian content), but the listing lacks details on seniority, location, and contract type, making it hard to fully assess fit.</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t>No location specified; if this is a UN consultancy based in Switzerland, it would be excluded per candidate preferences.</t>
         </is>
@@ -530,28 +546,33 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
           <t>Planning Officer</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>MONUSCO - United Nations Organisation Stabilization Mission in the Democratic Republic of the Congo</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="D4" t="inlineStr">
         <is>
           <t>https://untalent.org/jobs/planning-officer-23</t>
         </is>
       </c>
-      <c r="D4" t="n">
+      <c r="E4" t="n">
         <v>0.03</v>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="F4" t="inlineStr">
         <is>
           <t>Planning Officer role for MONUSCO in DRC has no alignment with candidate's multimedia/video production and communications background, target titles, or priority locations.</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="G4" t="inlineStr">
         <is>
           <t>DRC not in candidate's location list; likely UN field mission contract requiring separate visa/status arrangements.</t>
         </is>
@@ -560,28 +581,33 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
           <t>Associate External Relations Officer</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="C5" t="inlineStr">
         <is>
           <t>UNHCR - UN High Commissioner for Refugees</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="D5" t="inlineStr">
         <is>
           <t>https://untalent.org/jobs/associate-external-relations-officer-21</t>
         </is>
       </c>
-      <c r="D5" t="n">
+      <c r="E5" t="n">
         <v>0.25</v>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="F5" t="inlineStr">
         <is>
           <t>Title 'Associate External Relations Officer' is only tangentially related to target roles (communications-adjacent but not video/multimedia production focused), and likely UN-affiliated which may fall under excluded contract types.</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="G5" t="inlineStr">
         <is>
           <t>Location not specified in listing; if Switzerland-based UN role, may fall under excluded 'UN consultancy based in Switzerland' contract type.</t>
         </is>
@@ -590,132 +616,153 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
           <t>Finance Officer</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="C6" t="inlineStr">
         <is>
           <t>WVI - World Vision International</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="D6" t="inlineStr">
         <is>
           <t>https://untalent.org/jobs/finance-officer-504</t>
         </is>
       </c>
-      <c r="D6" t="n">
+      <c r="E6" t="n">
         <v>0.02</v>
       </c>
-      <c r="E6" t="inlineStr">
+      <c r="F6" t="inlineStr">
         <is>
           <t>Finance Officer role has no overlap with candidate's multimedia/production and communications skill set or target titles.</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
           <t>Fundraising Communications Intern (French-speaking)</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="C7" t="inlineStr">
         <is>
           <t>UNHCR - UN High Commissioner for Refugees</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="D7" t="inlineStr">
         <is>
           <t>https://untalent.org/jobs/fundraising-communications-intern-french-speaking-3</t>
         </is>
       </c>
-      <c r="D7" t="n">
+      <c r="E7" t="n">
         <v>0.05</v>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="F7" t="inlineStr">
         <is>
           <t>This is an internship position, explicitly excluded by the candidate's profile which targets mid-level roles and excludes internships.</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
           <t>MHPSS Officer</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="C8" t="inlineStr">
         <is>
           <t>Save the Children</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="D8" t="inlineStr">
         <is>
           <t>https://untalent.org/jobs/mhpss-officer-18</t>
         </is>
       </c>
-      <c r="D8" t="n">
+      <c r="E8" t="n">
         <v>0.02</v>
       </c>
-      <c r="E8" t="inlineStr">
+      <c r="F8" t="inlineStr">
         <is>
           <t>MHPSS Officer is a mental health/psychosocial support role, entirely unrelated to multimedia production, video editing, or communications skill set of the candidate.</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
           <t>MHPSS Officer (Maternity Cover)</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="C9" t="inlineStr">
         <is>
           <t>Save the Children</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="D9" t="inlineStr">
         <is>
           <t>https://untalent.org/jobs/mhpss-officer-maternity-cover</t>
         </is>
       </c>
-      <c r="D9" t="n">
+      <c r="E9" t="n">
         <v>0.05</v>
       </c>
-      <c r="E9" t="inlineStr">
+      <c r="F9" t="inlineStr">
         <is>
           <t>MHPSS (mental health/psychosocial support) Officer role is unrelated to video/multimedia production or communications skillset in the profile.</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
           <t>Programme Management Officer, Administration</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="C10" t="inlineStr">
         <is>
           <t>BINUH - United Nations Mission Integrated Office in Haiti</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="D10" t="inlineStr">
         <is>
           <t>https://untalent.org/jobs/programme-management-officer-administration-70</t>
         </is>
       </c>
-      <c r="D10" t="n">
+      <c r="E10" t="n">
         <v>0.03</v>
       </c>
-      <c r="E10" t="inlineStr">
+      <c r="F10" t="inlineStr">
         <is>
           <t>Programme Management Officer, Administration role in Haiti has no alignment with candidate's multimedia/video production and communications background, and Haiti is not among priority, secondary, or stretch locations.</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr">
+      <c r="G10" t="inlineStr">
         <is>
           <t>Location (Haiti) not in candidate's location preferences; visa/sponsorship relevance unclear but irrelevant given mismatch.</t>
         </is>
@@ -724,28 +771,33 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
           <t>Content Experience Manager</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="C11" t="inlineStr">
         <is>
           <t>ewz</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="D11" t="inlineStr">
         <is>
           <t>https://www.jobup.ch/en/jobs/detail/4c700729-c932-400d-a4e0-0902ae31e202/</t>
         </is>
       </c>
-      <c r="D11" t="n">
+      <c r="E11" t="n">
         <v>0.15</v>
       </c>
-      <c r="E11" t="inlineStr">
+      <c r="F11" t="inlineStr">
         <is>
           <t>Title 'Content Experience Manager' at a Swiss utility (ewz) doesn't align with target multimedia/video production or communications roles, and lacks details on humanitarian/social storytelling focus.</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr">
+      <c r="G11" t="inlineStr">
         <is>
           <t>Likely based in Zurich, Switzerland; as an EU/EEA citizen, no sponsorship needed.</t>
         </is>
@@ -754,106 +806,123 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
           <t>Junior Business Risk Officer (4 months - temporary contract)</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="C12" t="inlineStr">
         <is>
           <t>Swissquote Bank SA</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="D12" t="inlineStr">
         <is>
           <t>https://www.jobup.ch/en/jobs/detail/6e770285-aaf0-4ce8-9a16-315c672302f6/</t>
         </is>
       </c>
-      <c r="D12" t="n">
+      <c r="E12" t="n">
         <v>0</v>
       </c>
-      <c r="E12" t="inlineStr">
+      <c r="F12" t="inlineStr">
         <is>
           <t>Junior Business Risk Officer is unrelated to multimedia/video production or communications, is explicitly junior/temporary (excluded), and doesn't match any target titles or core skills.</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
           <t>Data Protection &amp; Privacy Specialist</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="C13" t="inlineStr">
         <is>
           <t>SICPA SA</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="D13" t="inlineStr">
         <is>
           <t>https://www.jobup.ch/en/jobs/detail/0f8707e3-bf8d-4466-9555-3ddcdceaaff4/</t>
         </is>
       </c>
-      <c r="D13" t="n">
+      <c r="E13" t="n">
         <v>0.03</v>
       </c>
-      <c r="E13" t="inlineStr">
+      <c r="F13" t="inlineStr">
         <is>
           <t>Data Protection &amp; Privacy Specialist role is entirely unrelated to the candidate's multimedia production, journalism, and communications background.</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
           <t>HR Officer (Fixed-term contract of 6M)</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="C14" t="inlineStr">
         <is>
           <t>Banque Pictet &amp; Cie SA</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
+      <c r="D14" t="inlineStr">
         <is>
           <t>https://www.jobup.ch/en/jobs/detail/775de108-25b9-4a69-b319-43423d60bb37/</t>
         </is>
       </c>
-      <c r="D14" t="n">
+      <c r="E14" t="n">
         <v>0.02</v>
       </c>
-      <c r="E14" t="inlineStr">
+      <c r="F14" t="inlineStr">
         <is>
           <t>HR Officer role has no relation to multimedia production, video, or communications skills in the candidate profile; completely different field.</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
           <t>Learning &amp; Talent Development Operations Officer (Fixed-term contract of 6M)</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
+      <c r="C15" t="inlineStr">
         <is>
           <t>Banque Pictet &amp; Cie SA</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
+      <c r="D15" t="inlineStr">
         <is>
           <t>https://www.jobup.ch/en/jobs/detail/92f04624-ddd4-476b-829d-b7f99a000663/</t>
         </is>
       </c>
-      <c r="D15" t="n">
+      <c r="E15" t="n">
         <v>0.02</v>
       </c>
-      <c r="E15" t="inlineStr">
+      <c r="F15" t="inlineStr">
         <is>
           <t>HR/Learning &amp; Talent Development role with no overlap in multimedia, video production, or communications skills; not aligned with target titles or core skills.</t>
         </is>
       </c>
-      <c r="F15" t="inlineStr">
+      <c r="G15" t="inlineStr">
         <is>
           <t>Switzerland-based (Geneva area likely); candidate is Polish/EU/EEA so no sponsorship needed, but role itself is irrelevant.</t>
         </is>

</xml_diff>

<commit_message>
Raise the match bar and add deadline/direct-link fields
- Only keep and remember listings scoring >= 0.4; below-threshold
  listings are discarded rather than shown or remembered, so they're
  re-evaluated (not permanently ignored) next run.
- Each fetcher now reports a deadline where the source provides one
  (ReliefWeb's date.closing, UN Talent's "N days left" converted to a
  date, IUCN's listed closing date; jobup.ch's API has no such field).
- Renames the URL column to Direct Link and adds Deadline, migrating
  the existing workbook rather than losing history.
</commit_message>
<xml_diff>
--- a/This_Weeks_Picks.xlsx
+++ b/This_Weeks_Picks.xlsx
@@ -424,16 +424,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G15"/>
+  <dimension ref="A1:H15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
     <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="45" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="55" customWidth="1" min="6" max="6"/>
-    <col width="30" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="45" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="55" customWidth="1" min="7" max="7"/>
+    <col width="30" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -454,20 +455,25 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>URL</t>
+          <t>Deadline</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
+          <t>Direct Link</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
           <t>Match Score</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Legal Work Flag</t>
         </is>
@@ -489,20 +495,20 @@
           <t>UNFPA - United Nations Population Fund</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>https://untalent.org/jobs/digital-content-creation-support-for-unfpa-campaigns-1</t>
         </is>
       </c>
-      <c r="E2" t="n">
+      <c r="F2" t="n">
         <v>0.55</v>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>Digital content creation for UNFPA campaigns aligns well with core skills (video production, social-first storytelling, humanitarian content) but title/location/contract type are unclear, and it may be a UN consultancy which is excluded if Switzerland-based.</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>Location not specified; if UN consultancy is based in Switzerland, this would be excluded per candidate preferences.</t>
         </is>
@@ -524,20 +530,20 @@
           <t>UNFPA - United Nations Population Fund</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="E3" t="inlineStr">
         <is>
           <t>https://untalent.org/jobs/digital-content-creation-support-for-unfpa-campaigns</t>
         </is>
       </c>
-      <c r="E3" t="n">
+      <c r="F3" t="n">
         <v>0.55</v>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t>Digital content creation for UNFPA campaigns aligns well with core skills (video production, social-first storytelling, humanitarian content), but the listing lacks details on seniority, location, and contract type, making it hard to fully assess fit.</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="H3" t="inlineStr">
         <is>
           <t>No location specified; if this is a UN consultancy based in Switzerland, it would be excluded per candidate preferences.</t>
         </is>
@@ -559,20 +565,20 @@
           <t>MONUSCO - United Nations Organisation Stabilization Mission in the Democratic Republic of the Congo</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="E4" t="inlineStr">
         <is>
           <t>https://untalent.org/jobs/planning-officer-23</t>
         </is>
       </c>
-      <c r="E4" t="n">
+      <c r="F4" t="n">
         <v>0.03</v>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="G4" t="inlineStr">
         <is>
           <t>Planning Officer role for MONUSCO in DRC has no alignment with candidate's multimedia/video production and communications background, target titles, or priority locations.</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="H4" t="inlineStr">
         <is>
           <t>DRC not in candidate's location list; likely UN field mission contract requiring separate visa/status arrangements.</t>
         </is>
@@ -594,20 +600,20 @@
           <t>UNHCR - UN High Commissioner for Refugees</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="E5" t="inlineStr">
         <is>
           <t>https://untalent.org/jobs/associate-external-relations-officer-21</t>
         </is>
       </c>
-      <c r="E5" t="n">
+      <c r="F5" t="n">
         <v>0.25</v>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="G5" t="inlineStr">
         <is>
           <t>Title 'Associate External Relations Officer' is only tangentially related to target roles (communications-adjacent but not video/multimedia production focused), and likely UN-affiliated which may fall under excluded contract types.</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
+      <c r="H5" t="inlineStr">
         <is>
           <t>Location not specified in listing; if Switzerland-based UN role, may fall under excluded 'UN consultancy based in Switzerland' contract type.</t>
         </is>
@@ -629,15 +635,15 @@
           <t>WVI - World Vision International</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="E6" t="inlineStr">
         <is>
           <t>https://untalent.org/jobs/finance-officer-504</t>
         </is>
       </c>
-      <c r="E6" t="n">
+      <c r="F6" t="n">
         <v>0.02</v>
       </c>
-      <c r="F6" t="inlineStr">
+      <c r="G6" t="inlineStr">
         <is>
           <t>Finance Officer role has no overlap with candidate's multimedia/production and communications skill set or target titles.</t>
         </is>
@@ -659,15 +665,15 @@
           <t>UNHCR - UN High Commissioner for Refugees</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="E7" t="inlineStr">
         <is>
           <t>https://untalent.org/jobs/fundraising-communications-intern-french-speaking-3</t>
         </is>
       </c>
-      <c r="E7" t="n">
+      <c r="F7" t="n">
         <v>0.05</v>
       </c>
-      <c r="F7" t="inlineStr">
+      <c r="G7" t="inlineStr">
         <is>
           <t>This is an internship position, explicitly excluded by the candidate's profile which targets mid-level roles and excludes internships.</t>
         </is>
@@ -689,15 +695,15 @@
           <t>Save the Children</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="E8" t="inlineStr">
         <is>
           <t>https://untalent.org/jobs/mhpss-officer-18</t>
         </is>
       </c>
-      <c r="E8" t="n">
+      <c r="F8" t="n">
         <v>0.02</v>
       </c>
-      <c r="F8" t="inlineStr">
+      <c r="G8" t="inlineStr">
         <is>
           <t>MHPSS Officer is a mental health/psychosocial support role, entirely unrelated to multimedia production, video editing, or communications skill set of the candidate.</t>
         </is>
@@ -719,15 +725,15 @@
           <t>Save the Children</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
+      <c r="E9" t="inlineStr">
         <is>
           <t>https://untalent.org/jobs/mhpss-officer-maternity-cover</t>
         </is>
       </c>
-      <c r="E9" t="n">
+      <c r="F9" t="n">
         <v>0.05</v>
       </c>
-      <c r="F9" t="inlineStr">
+      <c r="G9" t="inlineStr">
         <is>
           <t>MHPSS (mental health/psychosocial support) Officer role is unrelated to video/multimedia production or communications skillset in the profile.</t>
         </is>
@@ -749,20 +755,20 @@
           <t>BINUH - United Nations Mission Integrated Office in Haiti</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="E10" t="inlineStr">
         <is>
           <t>https://untalent.org/jobs/programme-management-officer-administration-70</t>
         </is>
       </c>
-      <c r="E10" t="n">
+      <c r="F10" t="n">
         <v>0.03</v>
       </c>
-      <c r="F10" t="inlineStr">
+      <c r="G10" t="inlineStr">
         <is>
           <t>Programme Management Officer, Administration role in Haiti has no alignment with candidate's multimedia/video production and communications background, and Haiti is not among priority, secondary, or stretch locations.</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr">
+      <c r="H10" t="inlineStr">
         <is>
           <t>Location (Haiti) not in candidate's location preferences; visa/sponsorship relevance unclear but irrelevant given mismatch.</t>
         </is>
@@ -784,20 +790,20 @@
           <t>ewz</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
+      <c r="E11" t="inlineStr">
         <is>
           <t>https://www.jobup.ch/en/jobs/detail/4c700729-c932-400d-a4e0-0902ae31e202/</t>
         </is>
       </c>
-      <c r="E11" t="n">
+      <c r="F11" t="n">
         <v>0.15</v>
       </c>
-      <c r="F11" t="inlineStr">
+      <c r="G11" t="inlineStr">
         <is>
           <t>Title 'Content Experience Manager' at a Swiss utility (ewz) doesn't align with target multimedia/video production or communications roles, and lacks details on humanitarian/social storytelling focus.</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr">
+      <c r="H11" t="inlineStr">
         <is>
           <t>Likely based in Zurich, Switzerland; as an EU/EEA citizen, no sponsorship needed.</t>
         </is>
@@ -819,15 +825,15 @@
           <t>Swissquote Bank SA</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
+      <c r="E12" t="inlineStr">
         <is>
           <t>https://www.jobup.ch/en/jobs/detail/6e770285-aaf0-4ce8-9a16-315c672302f6/</t>
         </is>
       </c>
-      <c r="E12" t="n">
+      <c r="F12" t="n">
         <v>0</v>
       </c>
-      <c r="F12" t="inlineStr">
+      <c r="G12" t="inlineStr">
         <is>
           <t>Junior Business Risk Officer is unrelated to multimedia/video production or communications, is explicitly junior/temporary (excluded), and doesn't match any target titles or core skills.</t>
         </is>
@@ -849,15 +855,15 @@
           <t>SICPA SA</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
+      <c r="E13" t="inlineStr">
         <is>
           <t>https://www.jobup.ch/en/jobs/detail/0f8707e3-bf8d-4466-9555-3ddcdceaaff4/</t>
         </is>
       </c>
-      <c r="E13" t="n">
+      <c r="F13" t="n">
         <v>0.03</v>
       </c>
-      <c r="F13" t="inlineStr">
+      <c r="G13" t="inlineStr">
         <is>
           <t>Data Protection &amp; Privacy Specialist role is entirely unrelated to the candidate's multimedia production, journalism, and communications background.</t>
         </is>
@@ -879,15 +885,15 @@
           <t>Banque Pictet &amp; Cie SA</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr">
+      <c r="E14" t="inlineStr">
         <is>
           <t>https://www.jobup.ch/en/jobs/detail/775de108-25b9-4a69-b319-43423d60bb37/</t>
         </is>
       </c>
-      <c r="E14" t="n">
+      <c r="F14" t="n">
         <v>0.02</v>
       </c>
-      <c r="F14" t="inlineStr">
+      <c r="G14" t="inlineStr">
         <is>
           <t>HR Officer role has no relation to multimedia production, video, or communications skills in the candidate profile; completely different field.</t>
         </is>
@@ -909,20 +915,20 @@
           <t>Banque Pictet &amp; Cie SA</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr">
+      <c r="E15" t="inlineStr">
         <is>
           <t>https://www.jobup.ch/en/jobs/detail/92f04624-ddd4-476b-829d-b7f99a000663/</t>
         </is>
       </c>
-      <c r="E15" t="n">
+      <c r="F15" t="n">
         <v>0.02</v>
       </c>
-      <c r="F15" t="inlineStr">
+      <c r="G15" t="inlineStr">
         <is>
           <t>HR/Learning &amp; Talent Development role with no overlap in multimedia, video production, or communications skills; not aligned with target titles or core skills.</t>
         </is>
       </c>
-      <c r="G15" t="inlineStr">
+      <c r="H15" t="inlineStr">
         <is>
           <t>Switzerland-based (Geneva area likely); candidate is Polish/EU/EEA so no sponsorship needed, but role itself is irrelevant.</t>
         </is>

</xml_diff>

<commit_message>
Weekly job search run - 2026-08-10
</commit_message>
<xml_diff>
--- a/This_Weeks_Picks.xlsx
+++ b/This_Weeks_Picks.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H15"/>
+  <dimension ref="A1:H18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -934,6 +934,126 @@
         </is>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Communications Officer (P)</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>IOM</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>https://fa-evlj-saasfaprod1.fa.ocs.oraclecloud.com/hcmUI/CandidateExperience/en/sites/CX_1001/job/21881</t>
+        </is>
+      </c>
+      <c r="F16" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Title directly matches target 'Communications Officer' and IOM is a global affairs/humanitarian organization, but the listing lacks location, seniority, and skill details needed to confirm fit.</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>No location specified; if Switzerland-based UN staff (not consultancy), sponsorship may still be required depending on nationality quotas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Media and Communications Officer (P)</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>IOM</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>https://fa-evlj-saasfaprod1.fa.ocs.oraclecloud.com/hcmUI/CandidateExperience/en/sites/CX_1001/job/21831</t>
+        </is>
+      </c>
+      <c r="F17" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Title 'Media and Communications Officer' aligns well with target titles and IOM humanitarian focus fits core skills, but listing lacks location/seniority/contract details needed to confirm fit, and IOM roles are often UN-affiliated positions that may resemble excluded consultancy types.</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>No location specified in listing; if Switzerland-based UN consultancy, would be excluded per candidate preferences.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Communications Officer (P)</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>IOM</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>https://fa-evlj-saasfaprod1.fa.ocs.oraclecloud.com/hcmUI/CandidateExperience/en/sites/CX_1001/job/22335</t>
+        </is>
+      </c>
+      <c r="F18" t="n">
+        <v>0.72</v>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Exact title match (Communications Officer) at IOM, a humanitarian/global affairs organization aligning with core skills; P-grade suggests professional/mid-level role, but listing lacks location and detailed requirements for full assessment.</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>No location specified in listing; visa/sponsorship relevance cannot be determined.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Weekly job search run - 2026-08-31
</commit_message>
<xml_diff>
--- a/This_Weeks_Picks.xlsx
+++ b/This_Weeks_Picks.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H18"/>
+  <dimension ref="A1:H19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1054,6 +1054,41 @@
         </is>
       </c>
     </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Private Sector Communications Officer</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>UNHCR</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>https://unhcr.wd3.myworkdayjobs.com/en-US/External/job/Bangkok-GlobProg-Thailand/Private-Sector-Communications-Officer_JR2668507</t>
+        </is>
+      </c>
+      <c r="F19" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Title matches target 'Communications Officer' and is mid-level, but the role focuses on private sector partnership communications rather than video/multimedia production; location (Bangkok) is a stretch location, not core skill area.</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Bangkok location; visa sponsorship likely required as candidate is Polish/EU, no local work authorization implied.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Weekly job search run - 2026-09-07
</commit_message>
<xml_diff>
--- a/This_Weeks_Picks.xlsx
+++ b/This_Weeks_Picks.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H19"/>
+  <dimension ref="A1:H21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1089,6 +1089,77 @@
         </is>
       </c>
     </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Communications and Advocacy Officer (Climate Resilience Project)</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Plan International</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>https://untalent.org/jobs/communications-and-advocacy-officer-climate-resilience-project</t>
+        </is>
+      </c>
+      <c r="F20" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>Title aligns with 'Communications Officer' target but focuses on advocacy/climate resilience rather than multimedia/video production core skills; location and seniority level unspecified.</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Media and Communications Officer (P)</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>IOM</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>https://fa-evlj-saasfaprod1.fa.ocs.oraclecloud.com/hcmUI/CandidateExperience/en/sites/CX_1001/job/22673</t>
+        </is>
+      </c>
+      <c r="F21" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>Title aligns with Communications Officer target and IOM is humanitarian/global affairs relevant, but listing lacks location, seniority (P-grade may be entry/mid professional UN track), and specific video/multimedia production details needed to confirm fit.</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>No location specified; if outside EU/EEA sponsorship status unclear, and if Switzerland-based UN role may fall under excluded consultancy type (though this appears to be a staff position, not consultancy).</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Weekly job search run - 2026-09-21
</commit_message>
<xml_diff>
--- a/This_Weeks_Picks.xlsx
+++ b/This_Weeks_Picks.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H21"/>
+  <dimension ref="A1:H22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1159,6 +1159,41 @@
         </is>
       </c>
     </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Multimedia Producer – Video, Motion Design &amp; Virtual Reality (80-100%)</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>IWF AG</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>https://www.jobup.ch/en/jobs/detail/ef27b869-32ee-4629-9f3b-3904a28cda41/</t>
+        </is>
+      </c>
+      <c r="F22" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>Title matches 'Multimedia Producer' and is likely Switzerland-based (priority location), but the role's heavy focus on motion design and VR diverges from the candidate's core social-first/humanitarian video storytelling skill set.</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>Switzerland-based role; as an EU/EEA (Polish) citizen, no visa sponsorship needed.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Weekly job search run - 2026-09-28
</commit_message>
<xml_diff>
--- a/This_Weeks_Picks.xlsx
+++ b/This_Weeks_Picks.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H22"/>
+  <dimension ref="A1:H23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1194,6 +1194,41 @@
         </is>
       </c>
     </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Digital Communications &amp; Marketing Officer (maternity cover)JRS - Jesuit Refugee ServiceRomeMid - Mid level</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>JRS - Jesuit Refugee Service</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>https://www.impactpool.org/jobs/1238556</t>
+        </is>
+      </c>
+      <c r="F23" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>Title partially aligns with target 'Communications Officer' and is mid-level, but focuses more on digital marketing/communications than video/multimedia production; Rome falls under secondary 'Europe' location.</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>EU/EEA citizenship should allow work in Italy without sponsorship.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Weekly job search run - 2026-10-05
</commit_message>
<xml_diff>
--- a/This_Weeks_Picks.xlsx
+++ b/This_Weeks_Picks.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H23"/>
+  <dimension ref="A1:H24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1229,6 +1229,46 @@
         </is>
       </c>
     </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Media and Communications Officer (P)</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>IOM</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>https://fa-evlj-saasfaprod1.fa.ocs.oraclecloud.com/hcmUI/CandidateExperience/en/sites/CX_1001/job/23233</t>
+        </is>
+      </c>
+      <c r="F24" t="n">
+        <v>0.62</v>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>Title directly matches target role (Communications Officer) and IOM is a strong humanitarian/global affairs fit, but listing lacks location details and seniority (P-grade) could skew above mid-level, requiring verification.</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>Location not specified in listing; if Switzerland-based UN consultancy, would be excluded per candidate's contract preferences.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Weekly job search run - 2026-10-12
</commit_message>
<xml_diff>
--- a/This_Weeks_Picks.xlsx
+++ b/This_Weeks_Picks.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H24"/>
+  <dimension ref="A1:H25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1269,6 +1269,41 @@
         </is>
       </c>
     </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>NGT Communications Officer (IT-CE-CHT-2026-242-GRAE)</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>CERN European Organization for Nuclear Research</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>https://www.jobup.ch/en/jobs/detail/17ec7d6c-8bd1-4c1e-8ef4-94f89f24698b/</t>
+        </is>
+      </c>
+      <c r="F25" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>Title matches target 'Communications Officer' and location (Geneva/CERN) is a top priority, but the listing gives no detail on video/multimedia production scope, making fit uncertain.</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>Geneva/CERN role - as an international organization CERN typically issues its own legitimation cards, so standard Swiss work visa rules may not apply; verify sponsorship/eligibility specifics.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>